<commit_message>
feat: add activate turn combat instruction and related functionality
- Implemented the `activateTurnCombat` instruction in the Solana program.
- Created TypeScript definitions and utility functions for the instruction.
- Added battle balance simulation and reporting features.
- Developed a WebSocket server for real-time battle interactions.
- Introduced hooks for managing battle room state in the client.
- Added tests for battle balance functionality.
</commit_message>
<xml_diff>
--- a/outputs/simultaneous-combat-backlog-20260911/WildQuest-Simultaneous-Turn-Combat-Backlog.xlsx
+++ b/outputs/simultaneous-combat-backlog-20260911/WildQuest-Simultaneous-Turn-Combat-Backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="1" r:id="R92ef1b4b6dd64e6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combat Rules" sheetId="2" r:id="Ra4e2047632ae4947"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UX and Sync" sheetId="3" r:id="Rd3ec410688984f59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Tests" sheetId="4" r:id="Rf62b4b6773ed45c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="1" r:id="R0114b3046df040ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combat Rules" sheetId="2" r:id="R2b847f42d2b9456e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UX and Sync" sheetId="3" r:id="R89fbeb3d5beb4f37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Tests" sheetId="4" r:id="R2a22e89741694462"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -960,7 +960,7 @@
       </x:c>
       <x:c r="B9" s="64" t="n">
         <x:f>COUNTIFS(I12:I60,"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C9" s="59"/>
       <x:c r="D9" s="35"/>
@@ -1089,7 +1089,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I12" s="67" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J12" s="67" t="str">
         <x:v>Yes</x:v>
@@ -1137,7 +1137,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I13" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J13" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1185,7 +1185,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I14" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J14" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1233,7 +1233,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I15" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J15" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1281,7 +1281,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I16" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J16" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1329,7 +1329,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I17" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J17" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1377,7 +1377,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I18" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J18" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1425,7 +1425,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I19" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J19" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1473,7 +1473,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I20" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J20" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1521,7 +1521,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I21" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J21" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1569,7 +1569,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I22" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J22" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1617,7 +1617,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I23" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J23" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1665,7 +1665,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I24" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J24" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1713,7 +1713,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I25" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J25" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1761,7 +1761,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I26" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J26" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1809,7 +1809,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I27" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J27" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1857,7 +1857,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I28" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J28" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1905,7 +1905,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I29" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J29" s="70" t="str">
         <x:v>Yes</x:v>
@@ -1953,7 +1953,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I30" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J30" s="70" t="str">
         <x:v>Yes</x:v>
@@ -2001,7 +2001,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I31" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J31" s="70" t="str">
         <x:v>Yes</x:v>
@@ -2049,7 +2049,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I32" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J32" s="70" t="str">
         <x:v>Yes</x:v>
@@ -2097,7 +2097,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I33" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J33" s="70" t="str">
         <x:v>Yes</x:v>
@@ -2145,7 +2145,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I34" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J34" s="70" t="str">
         <x:v>Yes</x:v>
@@ -2193,7 +2193,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I35" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J35" s="70" t="str">
         <x:v>Yes</x:v>
@@ -2241,7 +2241,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I36" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="J36" s="70" t="str">
         <x:v>Yes</x:v>
@@ -2289,7 +2289,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I37" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J37" s="70" t="str">
         <x:v>Yes</x:v>
@@ -2337,7 +2337,7 @@
         <x:v>MUST</x:v>
       </x:c>
       <x:c r="I38" s="70" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J38" s="70" t="str">
         <x:v>Yes</x:v>
@@ -8381,7 +8381,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb2479ce839941b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raded044d45b14cdc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9830,19 +9830,19 @@
         <x:v>Persian Cat</x:v>
       </x:c>
       <x:c r="C37" s="54" t="n">
-        <x:v>105</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="D37" s="54" t="n">
         <x:v>55</x:v>
       </x:c>
       <x:c r="E37" s="54" t="n">
-        <x:v>60</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="F37" s="54" t="n">
         <x:v>35</x:v>
       </x:c>
       <x:c r="G37" s="54" t="n">
-        <x:v>45</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="H37" s="78" t="n">
         <x:f>D37+INT(F37/5)</x:f>
@@ -23536,7 +23536,7 @@
         <x:v>Unit</x:v>
       </x:c>
       <x:c r="H7" s="53" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I7" s="1"/>
       <x:c r="J7" s="1"/>
@@ -23580,7 +23580,7 @@
         <x:v>Unit</x:v>
       </x:c>
       <x:c r="H8" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I8" s="1"/>
       <x:c r="J8" s="1"/>
@@ -23624,7 +23624,7 @@
         <x:v>Unit</x:v>
       </x:c>
       <x:c r="H9" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I9" s="1"/>
       <x:c r="J9" s="1"/>
@@ -23668,7 +23668,7 @@
         <x:v>Unit</x:v>
       </x:c>
       <x:c r="H10" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I10" s="1"/>
       <x:c r="J10" s="1"/>
@@ -23712,7 +23712,7 @@
         <x:v>Unit</x:v>
       </x:c>
       <x:c r="H11" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I11" s="1"/>
       <x:c r="J11" s="1"/>
@@ -23756,7 +23756,7 @@
         <x:v>Unit</x:v>
       </x:c>
       <x:c r="H12" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I12" s="1"/>
       <x:c r="J12" s="1"/>
@@ -23800,7 +23800,7 @@
         <x:v>Unit</x:v>
       </x:c>
       <x:c r="H13" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I13" s="1"/>
       <x:c r="J13" s="1"/>
@@ -23844,7 +23844,7 @@
         <x:v>Unit</x:v>
       </x:c>
       <x:c r="H14" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I14" s="1"/>
       <x:c r="J14" s="1"/>
@@ -23888,7 +23888,7 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="H15" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I15" s="1"/>
       <x:c r="J15" s="1"/>
@@ -23932,7 +23932,7 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="H16" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I16" s="1"/>
       <x:c r="J16" s="1"/>
@@ -23976,7 +23976,7 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="H17" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I17" s="1"/>
       <x:c r="J17" s="1"/>
@@ -24020,7 +24020,7 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="H18" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="I18" s="1"/>
       <x:c r="J18" s="1"/>
@@ -24064,7 +24064,7 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="H19" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I19" s="1"/>
       <x:c r="J19" s="1"/>
@@ -24108,7 +24108,7 @@
         <x:v>LiteSVM</x:v>
       </x:c>
       <x:c r="H20" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I20" s="1"/>
       <x:c r="J20" s="1"/>
@@ -24152,7 +24152,7 @@
         <x:v>LiteSVM</x:v>
       </x:c>
       <x:c r="H21" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I21" s="1"/>
       <x:c r="J21" s="1"/>
@@ -24196,7 +24196,7 @@
         <x:v>LiteSVM</x:v>
       </x:c>
       <x:c r="H22" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I22" s="1"/>
       <x:c r="J22" s="1"/>
@@ -24240,7 +24240,7 @@
         <x:v>LiteSVM</x:v>
       </x:c>
       <x:c r="H23" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I23" s="1"/>
       <x:c r="J23" s="1"/>
@@ -24284,7 +24284,7 @@
         <x:v>LiteSVM</x:v>
       </x:c>
       <x:c r="H24" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I24" s="1"/>
       <x:c r="J24" s="1"/>
@@ -24328,7 +24328,7 @@
         <x:v>Component</x:v>
       </x:c>
       <x:c r="H25" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I25" s="1"/>
       <x:c r="J25" s="1"/>
@@ -24372,7 +24372,7 @@
         <x:v>Component</x:v>
       </x:c>
       <x:c r="H26" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I26" s="1"/>
       <x:c r="J26" s="1"/>
@@ -24416,7 +24416,7 @@
         <x:v>Browser</x:v>
       </x:c>
       <x:c r="H27" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="I27" s="1"/>
       <x:c r="J27" s="1"/>
@@ -24460,7 +24460,7 @@
         <x:v>Browser</x:v>
       </x:c>
       <x:c r="H28" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="I28" s="1"/>
       <x:c r="J28" s="1"/>
@@ -24504,7 +24504,7 @@
         <x:v>Browser</x:v>
       </x:c>
       <x:c r="H29" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="I29" s="1"/>
       <x:c r="J29" s="1"/>
@@ -24548,7 +24548,7 @@
         <x:v>Simulation</x:v>
       </x:c>
       <x:c r="H30" s="54" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="I30" s="1"/>
       <x:c r="J30" s="1"/>
@@ -30748,7 +30748,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76ec92875b804a69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc18e43dbd8a840d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>